<commit_message>
Add agent inventory and decouple complexity profiles from models
</commit_message>
<xml_diff>
--- a/artifacts/custom-categories/custom-category-budget.xlsx
+++ b/artifacts/custom-categories/custom-category-budget.xlsx
@@ -40,7 +40,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Category usage'!$A$1:$F$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Category costs'!$A$1:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Monthly category summary'!$A$1:$H$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Profiles'!$A$1:$H$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Profiles'!$A$1:$G$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Scenarios'!$A$1:$G$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Additional costs'!$A$1:$A$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Pricing'!$A$1:$R$2</definedName>
@@ -2007,7 +2007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2017,7 +2017,6 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2056,11 +2055,6 @@
           <t>cache_write_fraction</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>model_id</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2098,11 +2092,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Category Fixture</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2140,7 +2129,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2178,7 +2166,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2216,14 +2203,9 @@
           <t>0</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Category Fixture</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H5"/>
+  <autoFilter ref="A1:G5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2555,7 +2537,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-04T01:29:12.897Z</t>
+          <t>2026-10-04T18:56:42.731Z</t>
         </is>
       </c>
       <c r="I2" s="2" t="b">
@@ -2820,7 +2802,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Schema 7; defaults 1</t>
+          <t>Schema 8; defaults 1</t>
         </is>
       </c>
     </row>
@@ -4769,7 +4751,11 @@
       <c r="D2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Category Fixture</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
@@ -4789,7 +4775,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>b6837f00-f73b-4494-b093-a33d4c7d07ad</t>
+          <t>d4d37538-c198-4e52-b943-40655bf87853</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -4891,7 +4877,11 @@
       <c r="D5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Category Fixture</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
@@ -4911,7 +4901,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>0097cb1e-f6e0-4cb1-aba0-0133e697dc3f</t>
+          <t>ee2a3270-28d1-454f-ab95-2c2f5f978ec0</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -4972,7 +4962,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>8956b06b-c919-4605-8090-79bec98cfb1a</t>
+          <t>7542484a-1920-41ab-954f-367b4f319a9e</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4982,7 +4972,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>b6837f00-f73b-4494-b093-a33d4c7d07ad</t>
+          <t>d4d37538-c198-4e52-b943-40655bf87853</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -4999,7 +4989,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>baa02f3a-986f-4516-90b2-8a62f201d2ab</t>
+          <t>d37dc99b-e13a-429d-b3d4-6e62b4545d4d</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5009,7 +4999,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0097cb1e-f6e0-4cb1-aba0-0133e697dc3f</t>
+          <t>ee2a3270-28d1-454f-ab95-2c2f5f978ec0</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -5155,7 +5145,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>8956b06b-c919-4605-8090-79bec98cfb1a</t>
+          <t>7542484a-1920-41ab-954f-367b4f319a9e</t>
         </is>
       </c>
     </row>
@@ -5200,7 +5190,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>689c9363-38bb-411b-9a4d-946a0ea2edac</t>
+          <t>e8ec7c95-429a-4c6d-8f9b-94e2b29e7d85</t>
         </is>
       </c>
     </row>
@@ -5245,7 +5235,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>18f90d0c-22cd-4582-bbf6-45aa17032bf4</t>
+          <t>9a898c20-7396-462e-812a-eec53deeca99</t>
         </is>
       </c>
     </row>
@@ -5290,7 +5280,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>baa02f3a-986f-4516-90b2-8a62f201d2ab</t>
+          <t>d37dc99b-e13a-429d-b3d4-6e62b4545d4d</t>
         </is>
       </c>
     </row>

</xml_diff>